<commit_message>
Removing Virtual envs for version controll
</commit_message>
<xml_diff>
--- a/app1/Excelfiles/2024wincandidates.xlsx
+++ b/app1/Excelfiles/2024wincandidates.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F545"/>
+  <dimension ref="A1:F559"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="24.88671875" customWidth="1" min="1" max="1"/>
@@ -15113,13 +15113,83 @@
       </c>
     </row>
     <row r="545">
-      <c r="A545" t="inlineStr"/>
-      <c r="B545" t="inlineStr"/>
-      <c r="C545" t="inlineStr"/>
-      <c r="D545" t="inlineStr"/>
-      <c r="E545" t="inlineStr"/>
       <c r="F545" t="n">
         <v>1</v>
+      </c>
+    </row>
+    <row r="546">
+      <c r="F546" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="547">
+      <c r="F547" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="548">
+      <c r="F548" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="549">
+      <c r="F549" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="550">
+      <c r="F550" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="551">
+      <c r="F551" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="552">
+      <c r="F552" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="553">
+      <c r="F553" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="554">
+      <c r="F554" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="555">
+      <c r="F555" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="556">
+      <c r="F556" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="557">
+      <c r="F557" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="558">
+      <c r="F558" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="559">
+      <c r="A559" t="inlineStr"/>
+      <c r="B559" t="inlineStr"/>
+      <c r="C559" t="inlineStr"/>
+      <c r="D559" t="inlineStr"/>
+      <c r="E559" t="inlineStr"/>
+      <c r="F559" t="n">
+        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>